<commit_message>
Altar Global Progression System (pt.1)
</commit_message>
<xml_diff>
--- a/Assets/StreamingAssets/Configs/Buildings/House.xlsx
+++ b/Assets/StreamingAssets/Configs/Buildings/House.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\IdleProject\Assets\StreamingAssets\Configs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\IdleProject\Assets\StreamingAssets\Configs\Buildings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CEFA458-D1D9-4F3D-BC67-F2E5A7D67D55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3E95263-F82B-4808-9863-A0290FC94855}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,9 +41,6 @@
   </si>
   <si>
     <t>worker_gold_cost</t>
-  </si>
-  <si>
-    <t>cumulative_gold_cost</t>
   </si>
   <si>
     <t>current_upgrade_level</t>
@@ -83,6 +80,9 @@
   </si>
   <si>
     <t>value</t>
+  </si>
+  <si>
+    <t>cumulative_worker_gold_cost</t>
   </si>
 </sst>
 </file>
@@ -369,7 +369,8 @@
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="4" width="21.88671875" customWidth="1"/>
+    <col min="3" max="3" width="28.77734375" customWidth="1"/>
+    <col min="4" max="4" width="21.88671875" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="17.109375" customWidth="1"/>
     <col min="10" max="10" width="24.44140625" customWidth="1"/>
@@ -383,7 +384,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="3"/>
@@ -4641,25 +4642,25 @@
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
@@ -19758,10 +19759,10 @@
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
@@ -19790,7 +19791,7 @@
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B2" s="4">
         <v>200</v>
@@ -19798,7 +19799,7 @@
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3" s="4">
         <v>1.1499999999999999</v>
@@ -19806,7 +19807,7 @@
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" s="4">
         <v>200</v>
@@ -19814,7 +19815,7 @@
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" s="4">
         <v>10</v>

</xml_diff>